<commit_message>
Add Tesla (TSLA) as cross-sector alternate
TSLA falls outside the original SaaS + Semiconductor framing, so it
joins as a 4th Alternate (selected=No) rather than reshuffling the 15
core names. Kept out of the weekly Monday/Tuesday/Wednesday rhythm
until a deliberate promotion decision.

Generated assets regenerated from generate_assets.py: company_universe
.csv, source_library.csv, google_alert_queries.csv, weekly_cadence.csv
and the Excel workbook (which now includes a TSLA company sheet via
selected_companies() — actually no, selected=No means it stays out of
sheet generation; only the universe row is added).

README Alternates line updated.
</commit_message>
<xml_diff>
--- a/data/CultureRadar_MVP_Workbook.xlsx
+++ b/data/CultureRadar_MVP_Workbook.xlsx
@@ -31,7 +31,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LRCX" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Company Universe'!$A$1:$P$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Company Universe'!$A$1:$P$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Judgment Tracker'!$A$1:$N$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Source Library'!$A$1:$H$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alert Queries'!$A$1:$G$91</definedName>
@@ -9153,7 +9153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -10476,16 +10476,86 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>TSLA</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Automotive / EV</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Electric vehicles / energy / autonomy</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Alternate</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Alternate (cross-sector)</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Cross-sector alternate. Huge public employee footprint, extreme management-language volatility, frequent talent inflows/outflows; no clean SaaS or semi peer, so kept as alternate rather than core.</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>Build baseline evidence log</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>Operational prioritization only; not a culture quality conclusion.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P19"/>
+  <autoFilter ref="A1:P20"/>
   <dataValidations count="3">
-    <dataValidation sqref="E2:E19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Core,Alternate"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M19" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Baseline complete,Ready to publish,Paused"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add TSMC (TSM) as cross-region alternate
Joins as a 5th Alternate (selected=No). TSMC fits the Semiconductor
industry label cleanly, so no new category needed. Kept out of the
weekly rhythm until a deliberate promotion decision.

README documents the methodological caveats: thin Western Glassdoor
sample (employee base mostly in Taiwan), low LinkedIn penetration of
TW engineers, bilingual transcripts requiring baseline-language
discipline before language-drift comparison.
</commit_message>
<xml_diff>
--- a/data/CultureRadar_MVP_Workbook.xlsx
+++ b/data/CultureRadar_MVP_Workbook.xlsx
@@ -31,7 +31,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LRCX" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Company Universe'!$A$1:$P$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Company Universe'!$A$1:$P$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Judgment Tracker'!$A$1:$N$51</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Source Library'!$A$1:$H$91</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Alert Queries'!$A$1:$G$91</definedName>
@@ -9153,7 +9153,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -10546,16 +10546,86 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>TSMC</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>TSM</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Semiconductor</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Pure-play foundry</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Alternate</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Alternate (cross-region)</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Cross-region alternate. World's leading pure-play foundry; heavy geopolitical and supply-chain narrative weight. Methodological caveats: Western Glassdoor sample is thin (employees mostly in Taiwan), LinkedIn penetration of TW engineers lower than US peers, transcripts bilingual (set baseline language before language-drift comparison).</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>Build baseline evidence log</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>Operational prioritization only; not a culture quality conclusion.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:P20"/>
+  <autoFilter ref="A1:P21"/>
   <dataValidations count="3">
-    <dataValidation sqref="E2:E20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Core,Alternate"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="M2:M21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,In progress,Baseline complete,Ready to publish,Paused"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>